<commit_message>
feat: add Kingdom support with per-kingdom Excel sheets and UI filtering
</commit_message>
<xml_diff>
--- a/data/Heroes.xlsx
+++ b/data/Heroes.xlsx
@@ -12,8 +12,16 @@
     <sheet name="Categories" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Roles" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Gods" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Heroes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Legacy_Export" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Kingdoms" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="K_Humans" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="K_Kingdom_of_Ores" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="K_Kingdom_of_Magic" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="K_Kingdom_of_Evil" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="K_Kingdom_of_the_Ancients" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="K_Kingdom_of_the_Beasts" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="K_Kingdom_of_the_Divines" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Heroes" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Legacy_Export" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,7 +450,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Age</t>
+          <t>Kingdom</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -459,7 +467,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Temple</t>
+          <t>Age</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -476,7 +484,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>God</t>
+          <t>Temple</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -493,7 +501,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hero Name</t>
+          <t>God</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -510,7 +518,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>Hero Name</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -527,12 +535,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Combat Stats</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -544,7 +552,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mobility</t>
+          <t>Health</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -561,7 +569,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Melee ATK</t>
+          <t>Mobility</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -578,7 +586,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ranged ATK</t>
+          <t>Melee ATK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -595,7 +603,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Magic ATK</t>
+          <t>Ranged ATK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,12 +620,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Melee DEF</t>
+          <t>Magic ATK</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>Combat Stats</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -629,7 +637,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ranged DEF</t>
+          <t>Melee DEF</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -646,7 +654,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Magic DEF</t>
+          <t>Ranged DEF</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -663,12 +671,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Healing</t>
+          <t>Magic DEF</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abilities</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -680,12 +688,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Melee Target Type</t>
+          <t>Healing</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Target Types</t>
+          <t>Abilities</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -697,7 +705,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ranged Target Type</t>
+          <t>Melee Target Type</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -714,7 +722,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Magical Target Type</t>
+          <t>Ranged Target Type</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -731,24 +739,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Passive</t>
+          <t>Magical Target Type</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Abilities</t>
+          <t>Target Types</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>textarea</t>
+          <t>text</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Abilities</t>
+          <t>Passive</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -765,7 +773,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ultimate Skill</t>
+          <t>Abilities</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -782,12 +790,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Ultimate Skill</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Custom</t>
+          <t>Abilities</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -799,29 +807,29 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Rage (Required to cast the Ultimate Skill)</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Resource</t>
+          <t>Custom</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>textarea</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Dodge</t>
+          <t>Rage (Required to cast the Ultimate Skill)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -833,7 +841,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Parry</t>
+          <t>Dodge</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -850,12 +858,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Speed</t>
+          <t>Parry</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Combat Stats</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -867,12 +875,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Speed</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Range &amp; AoE</t>
+          <t>Combat Stats</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -884,12 +892,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Armor</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Defense</t>
+          <t>Range &amp; AoE</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -901,12 +909,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cost</t>
+          <t>Armor</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Economy</t>
+          <t>Defense</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -918,7 +926,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Cost</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -935,15 +943,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>Area of Effect</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>Range &amp; AoE</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>text</t>
         </is>
@@ -954,47 +979,44 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Age</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Classical Age</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Medieval Age</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Mythic Age</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Sci-Mythic Age</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
         </is>
       </c>
     </row>
@@ -1003,82 +1025,44 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Category</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Abilities</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Combat Stats</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Defense</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Identity</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Range &amp; AoE</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Resource</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Target Types</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Custom</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
         </is>
       </c>
     </row>
@@ -1087,103 +1071,44 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Role</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Defensive Support</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Duelist</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Economy</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Elite Archer</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Fast Melee</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Frontline</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Heavy Cavalry</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Heavy Infantry</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Heavy Tank</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Ranged Unit</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Siege</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Support</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
         </is>
       </c>
     </row>
@@ -1192,40 +1117,44 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>God</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Athenia</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Barathor</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Ra</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1163,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1299,7 +1228,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{"Role": "Ranged Unit", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Ranged Unit", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Ranged Unit", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Ranged Unit", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1256,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{"Role": "Frontline", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Frontline", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Frontline", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Frontline", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1284,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{"Role": "Fast Melee", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Fast Melee", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Fast Melee", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Fast Melee", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1312,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{"Role": "Support", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "Healing", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Support", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "Healing", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1340,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Gather/Build", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Gather/Build", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1368,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{"Role": "Elite Archer", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Elite Archer", "God": "", "Temple": "None"}</t>
+          <t>{"Role": "Elite Archer", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Elite Archer", "God": "", "Temple": "None", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1396,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{"Role": "Heavy Infantry", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Heavy Infantry", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Heavy Infantry", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Heavy Infantry", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1495,7 +1424,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{"Role": "Support", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "Healing", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Support", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "Healing", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1452,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Food", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Food", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1480,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Construction", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Construction", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1508,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{"Role": "Siege", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Siege", "God": "", "Temple": ""}</t>
+          <t>{"Role": "Siege", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Siege", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1611,7 +1540,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>{"Role": "Infantry", "Health": "Extremely High", "Mobility": "Low-Moderate", "Melee ATK": "Very High", "Ranged ATK": "None", "Magic ATK": "Low (Holy attack)", "Melee DEF": "Extremely High", "Ranged DEF": "Moderately High", "Magic DEF": "Moderate", "Healing": "None", "Melee Target Type": "Melee Single Target", "Ranged Target Type": "None", "Magical Target Type": "AoE", "Passive": "Divine Retribution (Counterattack every hit)", "Abilities": "Heavy frontline tank", "Ultimate Skill": "Bulwark of Athenia: Increases the melee damage to a single target by 300%. AoE magical dmg to the enemy dmg factor 300 at exp lvl 5. After this skill is cast gains a massive damage absorption shield which absorbs dmg of 5000.", "Notes": "Strong vs Melee atatck, weaker vs Mages", "Rage (Required to cast the Ultimate Skill)": "1000", "Dodge": "High", "Parry": "Very High", "Speed": "", "Range": "", "Armor": "High", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Infantry", "God": "Athenia", "Temple": "Temple of Athenia"}</t>
+          <t>{"Role": "Infantry", "Health": "Extremely High", "Mobility": "Low-Moderate", "Melee ATK": "Very High", "Ranged ATK": "None", "Magic ATK": "Low (Holy attack)", "Melee DEF": "Extremely High", "Ranged DEF": "Moderately High", "Magic DEF": "Moderate", "Healing": "None", "Melee Target Type": "Melee Single Target", "Ranged Target Type": "None", "Magical Target Type": "AoE", "Passive": "Divine Retribution (Counterattack every hit)", "Abilities": "Heavy frontline tank", "Ultimate Skill": "Bulwark of Athenia: Increases the melee damage to a single target by 300%. AoE magical dmg to the enemy dmg factor 300 at exp lvl 5. After this skill is cast gains a massive damage absorption shield which absorbs dmg of 5000.", "Notes": "Strong vs Melee atatck, weaker vs Mages", "Rage (Required to cast the Ultimate Skill)": "1000", "Dodge": "High", "Parry": "Very High", "Speed": "", "Range": "", "Armor": "High", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Infantry", "God": "Athenia", "Temple": "Temple of Athenia", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1572,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>{"Role": "Support", "Health": "High", "Mobility": "Moderate", "Melee ATK": "Low", "Ranged ATK": "None", "Magic ATK": "Moderate", "Melee DEF": "Moderate", "Ranged DEF": "High", "Magic DEF": "Very High", "Healing": "AoE small healing.", "Melee Target Type": "Melee Single Target", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Prioritizes weakest Athenia hero", "Abilities": "Increase HP, Armor, Counterattack; Single-target anti-range &amp; anti-magic shield", "Ultimate Skill": "Shield of Athenia: Shields all ally heroes, reducing the dmg they receive by 2000. Prefers devotess of Athen first like Paldi. In case there is no Paladin then protects the hero wit least health first. Diesnt Protect the villagers or farmers.", "Notes": "No AoE healing", "Rage (Required to cast the Ultimate Skill)": "1000", "Dodge": "Very High", "Parry": "Very High", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "Athenia", "Temple": "Temple of Athenia"}</t>
+          <t>{"Role": "Support", "Health": "High", "Mobility": "Moderate", "Melee ATK": "Low", "Ranged ATK": "None", "Magic ATK": "Moderate", "Melee DEF": "Moderate", "Ranged DEF": "High", "Magic DEF": "Very High", "Healing": "AoE small healing.", "Melee Target Type": "Melee Single Target", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Prioritizes weakest Athenia hero", "Abilities": "Increase HP, Armor, Counterattack; Single-target anti-range &amp; anti-magic shield", "Ultimate Skill": "Shield of Athenia: Shields all ally heroes, reducing the dmg they receive by 2000. Prefers devotess of Athen first like Paldi. In case there is no Paladin then protects the hero wit least health first. Diesnt Protect the villagers or farmers.", "Notes": "No AoE healing", "Rage (Required to cast the Ultimate Skill)": "1000", "Dodge": "Very High", "Parry": "Very High", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "Athenia", "Temple": "Temple of Athenia", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1604,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{"Role": "Infantry", "Health": "Moderate", "Mobility": "High", "Melee ATK": "Extremely High", "Ranged ATK": "None", "Magic ATK": "Moderate (later levels)", "Melee DEF": "Moderate", "Ranged DEF": "Moderate", "Magic DEF": "Moderate", "Healing": "None", "Melee Target Type": "AoE (Whirlwind)", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Battle Focus", "Abilities": "Whirlwind Blades", "Ultimate Skill": "Barathor's Wrath: Does Single Target Damage of 5000 to a single target below exp lvl 5. At exp lvl 5 does AoE melee dmg upto 5 targets, dmg factor 5000, and brings whirlwind of blades increases dmg by 10% and reduce the rage requirement by 5%.", "Notes": "No lifesteal", "Rage (Required to cast the Ultimate Skill)": "800", "Dodge": "Very High", "Parry": "Moderate", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Infantry", "God": "Barathor", "Temple": "Temple of Barathor"}</t>
+          <t>{"Role": "Infantry", "Health": "Moderate", "Mobility": "High", "Melee ATK": "Extremely High", "Ranged ATK": "None", "Magic ATK": "Moderate (later levels)", "Melee DEF": "Moderate", "Ranged DEF": "Moderate", "Magic DEF": "Moderate", "Healing": "None", "Melee Target Type": "AoE (Whirlwind)", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Battle Focus", "Abilities": "Whirlwind Blades", "Ultimate Skill": "Barathor's Wrath: Does Single Target Damage of 5000 to a single target below exp lvl 5. At exp lvl 5 does AoE melee dmg upto 5 targets, dmg factor 5000, and brings whirlwind of blades increases dmg by 10% and reduce the rage requirement by 5%.", "Notes": "No lifesteal", "Rage (Required to cast the Ultimate Skill)": "800", "Dodge": "Very High", "Parry": "Moderate", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Infantry", "God": "Barathor", "Temple": "Temple of Barathor", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1636,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{"Role": "Support", "Health": "Moderate", "Mobility": "Moderate", "Melee ATK": "Low", "Ranged ATK": "None", "Magic ATK": "Moderate", "Melee DEF": "Low-Moderate", "Ranged DEF": "Moderate", "Magic DEF": "Moderate", "Healing": "Grants Lifesteal only to herself.", "Melee Target Type": "Single Target", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Aura: +10% Rage (Sword Master), +5% others", "Abilities": "Blood Pact, Battle Cry", "Ultimate Skill": "Blood Frenzy: Aura: +10% Rage (Sword Master), +5% others. At exp lvl 5, causes the dmg to enemy as life leech to heal herself.", "Notes": "Self gains lifesteal while enraged", "Rage (Required to cast the Ultimate Skill)": "900", "Dodge": "High", "Parry": "Moderate", "Speed": "Fast-Moderate", "Range": "", "Armor": "Moderate", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "Barathor", "Temple": "Temple of Barathor"}</t>
+          <t>{"Role": "Support", "Health": "Moderate", "Mobility": "Moderate", "Melee ATK": "Low", "Ranged ATK": "None", "Magic ATK": "Moderate", "Melee DEF": "Low-Moderate", "Ranged DEF": "Moderate", "Magic DEF": "Moderate", "Healing": "Grants Lifesteal only to herself.", "Melee Target Type": "Single Target", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Aura: +10% Rage (Sword Master), +5% others", "Abilities": "Blood Pact, Battle Cry", "Ultimate Skill": "Blood Frenzy: Aura: +10% Rage (Sword Master), +5% others. At exp lvl 5, causes the dmg to enemy as life leech to heal herself.", "Notes": "Self gains lifesteal while enraged", "Rage (Required to cast the Ultimate Skill)": "900", "Dodge": "High", "Parry": "Moderate", "Speed": "Fast-Moderate", "Range": "", "Armor": "Moderate", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "Barathor", "Temple": "Temple of Barathor", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1739,7 +1668,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{"Temple": "Temple to Ra", "God": "Ra", "Role": "War Commander", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "War Commander"}</t>
+          <t>{"Temple": "Temple to Ra", "God": "Ra", "Role": "War Commander", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "War Commander", "Kingdom": "Humans"}</t>
         </is>
       </c>
     </row>
@@ -1748,162 +1677,167 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD17"/>
+  <dimension ref="A1:AE17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Kingdom</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Temple</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>God</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Hero Name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Mobility</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Melee ATK</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Ranged ATK</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Magic ATK</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Melee DEF</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Ranged DEF</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Magic DEF</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Healing</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Melee Target Type</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Ranged Target Type</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Magical Target Type</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Passive</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Abilities</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Ultimate Skill</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Rage (Required to cast the Ultimate Skill)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Dodge</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Parry</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Speed</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Armor</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Population</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Area of Effect</t>
         </is>
@@ -1912,22 +1846,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Classical Age</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Archer</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Ranged Unit</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
@@ -1952,26 +1890,31 @@
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
       <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Classical Age</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Infantry</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Frontline</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
@@ -1996,26 +1939,31 @@
       <c r="AB3" t="inlineStr"/>
       <c r="AC3" t="inlineStr"/>
       <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Classical Age</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Cavalry</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Fast Melee</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
@@ -2040,26 +1988,31 @@
       <c r="AB4" t="inlineStr"/>
       <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Classical Age</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Healer</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
@@ -2067,12 +2020,12 @@
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
         <is>
           <t>Healing</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
@@ -2088,26 +2041,31 @@
       <c r="AB5" t="inlineStr"/>
       <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Classical Age</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Villager</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
@@ -2116,12 +2074,12 @@
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
         <is>
           <t>Gather/Build</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
@@ -2136,30 +2094,35 @@
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
       <c r="AD6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Medieval Age</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Ranger</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Elite Archer</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
@@ -2184,26 +2147,31 @@
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
       <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Medieval Age</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Knight</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Heavy Infantry</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
@@ -2228,26 +2196,31 @@
       <c r="AB8" t="inlineStr"/>
       <c r="AC8" t="inlineStr"/>
       <c r="AD8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Medieval Age</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Medic</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -2255,12 +2228,12 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
         <is>
           <t>Healing</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
@@ -2276,26 +2249,31 @@
       <c r="AB9" t="inlineStr"/>
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Medieval Age</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Farmer</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
@@ -2304,12 +2282,12 @@
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr">
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
         <is>
           <t>Food</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
@@ -2324,26 +2302,31 @@
       <c r="AB10" t="inlineStr"/>
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Medieval Age</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Builder</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>Economy</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -2352,12 +2335,12 @@
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr">
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
         <is>
           <t>Construction</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
@@ -2372,26 +2355,31 @@
       <c r="AB11" t="inlineStr"/>
       <c r="AC11" t="inlineStr"/>
       <c r="AD11" t="inlineStr"/>
+      <c r="AE11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Medieval Age</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Siege Units</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>Siege</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
@@ -2416,534 +2404,559 @@
       <c r="AB12" t="inlineStr"/>
       <c r="AC12" t="inlineStr"/>
       <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Mythic Age</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Temple of Athenia</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Athenia</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Paladin</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>Infantry</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Extremely High</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Low-Moderate</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Low (Holy attack)</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Extremely High</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Moderately High</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Melee Single Target</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
+      <c r="Q13" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="R13" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>Divine Retribution (Counterattack every hit)</t>
         </is>
       </c>
-      <c r="S13" t="inlineStr">
+      <c r="T13" t="inlineStr">
         <is>
           <t>Heavy frontline tank</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>Bulwark of Athenia: Increases the melee damage to a single target by 300%. AoE magical dmg to the enemy dmg factor 300 at exp lvl 5. After this skill is cast gains a massive damage absorption shield which absorbs dmg of 5000.</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>Strong vs Melee atatck, weaker vs Mages</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="W13" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="X13" t="inlineStr">
+      <c r="Y13" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr">
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr"/>
       <c r="AC13" t="inlineStr"/>
       <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>Mythic Age</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Temple of Athenia</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Athenia</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Guardian of Athenia</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
+      <c r="O14" t="inlineStr">
         <is>
           <t>AoE small healing.</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>Melee Single Target</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr">
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
         <is>
           <t>Prioritizes weakest Athenia hero</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>Increase HP, Armor, Counterattack; Single-target anti-range &amp; anti-magic shield</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>Shield of Athenia: Shields all ally heroes, reducing the dmg they receive by 2000. Prefers devotess of Athen first like Paldi. In case there is no Paladin then protects the hero wit least health first. Diesnt Protect the villagers or farmers.</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>No AoE healing</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="W14" t="inlineStr">
         <is>
           <t>1000</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
       </c>
-      <c r="X14" t="inlineStr">
+      <c r="Y14" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr"/>
       <c r="AB14" t="inlineStr"/>
       <c r="AC14" t="inlineStr"/>
       <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Mythic Age</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Temple of Barathor</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Barathor</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Sword Master</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>Infantry</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Extremely High</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="J15" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>Moderate (later levels)</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr">
+      <c r="O15" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>AoE (Whirlwind)</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr">
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
         <is>
           <t>Battle Focus</t>
         </is>
       </c>
-      <c r="S15" t="inlineStr">
+      <c r="T15" t="inlineStr">
         <is>
           <t>Whirlwind Blades</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="U15" t="inlineStr">
         <is>
           <t>Barathor's Wrath: Does Single Target Damage of 5000 to a single target below exp lvl 5. At exp lvl 5 does AoE melee dmg upto 5 targets, dmg factor 5000, and brings whirlwind of blades increases dmg by 10% and reduce the rage requirement by 5%.</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>No lifesteal</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="W15" t="inlineStr">
         <is>
           <t>800</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>Very High</t>
         </is>
       </c>
-      <c r="X15" t="inlineStr">
+      <c r="Y15" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr"/>
       <c r="AA15" t="inlineStr"/>
       <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr"/>
       <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>Mythic Age</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Temple of Barathor</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Barathor</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Priestess of Barathor</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="J16" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Low-Moderate</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>Grants Lifesteal only to herself.</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>Single Target</t>
         </is>
       </c>
-      <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr">
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
         <is>
           <t>Aura: +10% Rage (Sword Master), +5% others</t>
         </is>
       </c>
-      <c r="S16" t="inlineStr">
+      <c r="T16" t="inlineStr">
         <is>
           <t>Blood Pact, Battle Cry</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="U16" t="inlineStr">
         <is>
           <t>Blood Frenzy: Aura: +10% Rage (Sword Master), +5% others. At exp lvl 5, causes the dmg to enemy as life leech to heal herself.</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>Self gains lifesteal while enraged</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="W16" t="inlineStr">
         <is>
           <t>900</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="Y16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Z16" t="inlineStr">
         <is>
           <t>Fast-Moderate</t>
         </is>
       </c>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr">
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr"/>
       <c r="AC16" t="inlineStr"/>
       <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Humans</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>Sci-Mythic Age</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Temple to Ra</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Ra</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Son of Ra</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>War Commander</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
@@ -2968,6 +2981,963 @@
       <c r="AB17" t="inlineStr"/>
       <c r="AC17" t="inlineStr"/>
       <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Classical Age</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mythic Age</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sci-Mythic Age</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Abilities</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Combat Stats</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Range &amp; AoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Target Types</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Custom</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Defensive Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Duelist</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Elite Archer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fast Melee</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Frontline</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Heavy Cavalry</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Heavy Infantry</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Heavy Tank</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Ranged Unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Siege</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Support</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>God</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Athenia</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Barathor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ra</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Kingdom</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Humans</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Kingdom of Ores</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Kingdom of Magic</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Kingdom of Evil</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Kingdom of the Ancients</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Kingdom of the Beasts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kingdom of the Divines</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>771562e2-929a-4ef8-9afd-cc9859a09e55</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Classical Age</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Archer</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>{"Role": "Ranged Unit", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Ranged Unit", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>653c8feb-c0ef-4400-8d57-f60f5c1a5030</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Classical Age</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Infantry</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>{"Role": "Frontline", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Frontline", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>81cec51d-95ac-4544-980c-4084d4911af9</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Classical Age</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cavalry</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>{"Role": "Fast Melee", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Fast Melee", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>02ad382c-ba37-4428-b0b4-2261bcd6f427</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Classical Age</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Healer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>{"Role": "Support", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "Healing", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0b23742a-85e9-4eec-a7b6-7799107c6773</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Classical Age</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Villager</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Gather/Build", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ccb6d4bc-0e29-482a-8b71-924b9e1a59d8</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Ranger</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>{"Role": "Elite Archer", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Elite Archer", "God": "", "Temple": "None", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>be83df14-3c9e-4160-a028-8c63b8225495</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Knight</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>{"Role": "Heavy Infantry", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Heavy Infantry", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>de885831-0eed-4b07-b62b-c0d618be6a71</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Medic</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>{"Role": "Support", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "Healing", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2d1be3fe-d2bf-4f7c-bfc9-77a9c9acf4f5</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Farmer</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Food", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2c2c5251-3c6a-4ed9-9d92-333483031075</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Builder</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>{"Role": "Economy", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "Construction", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Economy", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>09048511-65ff-4f55-b485-e9b66390066d</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Medieval Age</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Siege Units</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>{"Role": "Siege", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Siege", "God": "", "Temple": "", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>b513bb4b-b84e-4000-96f4-27fcd108ffd7</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mythic Age</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Paladin</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>32827d776e6e45159ee75b44639f494b.png</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>{"Role": "Infantry", "Health": "Extremely High", "Mobility": "Low-Moderate", "Melee ATK": "Very High", "Ranged ATK": "None", "Magic ATK": "Low (Holy attack)", "Melee DEF": "Extremely High", "Ranged DEF": "Moderately High", "Magic DEF": "Moderate", "Healing": "None", "Melee Target Type": "Melee Single Target", "Ranged Target Type": "None", "Magical Target Type": "AoE", "Passive": "Divine Retribution (Counterattack every hit)", "Abilities": "Heavy frontline tank", "Ultimate Skill": "Bulwark of Athenia: Increases the melee damage to a single target by 300%. AoE magical dmg to the enemy dmg factor 300 at exp lvl 5. After this skill is cast gains a massive damage absorption shield which absorbs dmg of 5000.", "Notes": "Strong vs Melee atatck, weaker vs Mages", "Rage (Required to cast the Ultimate Skill)": "1000", "Dodge": "High", "Parry": "Very High", "Speed": "", "Range": "", "Armor": "High", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Infantry", "God": "Athenia", "Temple": "Temple of Athenia", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>81cc5b82-491f-4bc1-aec1-b8d32ba07f56</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Mythic Age</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Guardian of Athenia</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>d3cb5c4911324ed08a4d4b1db4c9b798.png</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>{"Role": "Support", "Health": "High", "Mobility": "Moderate", "Melee ATK": "Low", "Ranged ATK": "None", "Magic ATK": "Moderate", "Melee DEF": "Moderate", "Ranged DEF": "High", "Magic DEF": "Very High", "Healing": "AoE small healing.", "Melee Target Type": "Melee Single Target", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Prioritizes weakest Athenia hero", "Abilities": "Increase HP, Armor, Counterattack; Single-target anti-range &amp; anti-magic shield", "Ultimate Skill": "Shield of Athenia: Shields all ally heroes, reducing the dmg they receive by 2000. Prefers devotess of Athen first like Paldi. In case there is no Paladin then protects the hero wit least health first. Diesnt Protect the villagers or farmers.", "Notes": "No AoE healing", "Rage (Required to cast the Ultimate Skill)": "1000", "Dodge": "Very High", "Parry": "Very High", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "Athenia", "Temple": "Temple of Athenia", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>66035c9a-5564-4913-8594-d7956b114541</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mythic Age</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sword Master</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>9423cef7d7b2474bb3e85dd1fa1ce773.png</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>{"Role": "Infantry", "Health": "Moderate", "Mobility": "High", "Melee ATK": "Extremely High", "Ranged ATK": "None", "Magic ATK": "Moderate (later levels)", "Melee DEF": "Moderate", "Ranged DEF": "Moderate", "Magic DEF": "Moderate", "Healing": "None", "Melee Target Type": "AoE (Whirlwind)", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Battle Focus", "Abilities": "Whirlwind Blades", "Ultimate Skill": "Barathor's Wrath: Does Single Target Damage of 5000 to a single target below exp lvl 5. At exp lvl 5 does AoE melee dmg upto 5 targets, dmg factor 5000, and brings whirlwind of blades increases dmg by 10% and reduce the rage requirement by 5%.", "Notes": "No lifesteal", "Rage (Required to cast the Ultimate Skill)": "800", "Dodge": "Very High", "Parry": "Moderate", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Infantry", "God": "Barathor", "Temple": "Temple of Barathor", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>62b5c643-dc61-4c0b-a2d6-2f2651ff60fa</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Mythic Age</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Priestess of Barathor</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>f31eeb17a626474cba44a8753725f992.png</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>{"Role": "Support", "Health": "Moderate", "Mobility": "Moderate", "Melee ATK": "Low", "Ranged ATK": "None", "Magic ATK": "Moderate", "Melee DEF": "Low-Moderate", "Ranged DEF": "Moderate", "Magic DEF": "Moderate", "Healing": "Grants Lifesteal only to herself.", "Melee Target Type": "Single Target", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "Aura: +10% Rage (Sword Master), +5% others", "Abilities": "Blood Pact, Battle Cry", "Ultimate Skill": "Blood Frenzy: Aura: +10% Rage (Sword Master), +5% others. At exp lvl 5, causes the dmg to enemy as life leech to heal herself.", "Notes": "Self gains lifesteal while enraged", "Rage (Required to cast the Ultimate Skill)": "900", "Dodge": "High", "Parry": "Moderate", "Speed": "Fast-Moderate", "Range": "", "Armor": "Moderate", "Cost": "", "Population": "", "Area of Effect": "", "_type": "Support", "God": "Barathor", "Temple": "Temple of Barathor", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1008edc1-eb91-4f58-b0cf-23ab23f5d1d8</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Sci-Mythic Age</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Son of Ra</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>a7a08b0ad9f64b3bac9e98e815f76979.png</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>{"Temple": "Temple to Ra", "God": "Ra", "Role": "War Commander", "Health": "", "Mobility": "", "Melee ATK": "", "Ranged ATK": "", "Magic ATK": "", "Melee DEF": "", "Ranged DEF": "", "Magic DEF": "", "Healing": "", "Melee Target Type": "", "Ranged Target Type": "", "Magical Target Type": "", "Passive": "", "Abilities": "", "Ultimate Skill": "", "Notes": "", "Rage (Required to cast the Ultimate Skill)": "", "Dodge": "", "Parry": "", "Speed": "", "Range": "", "Armor": "", "Cost": "", "Population": "", "Area of Effect": "", "_type": "War Commander", "Kingdom": "Humans"}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Hero Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Portrait</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Extra Images</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data JSON</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>